<commit_message>
Update reviewed birthday corrections
</commit_message>
<xml_diff>
--- a/SNH48成员名单生日表2603 (1).xlsx
+++ b/SNH48成员名单生日表2603 (1).xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="4" r:id="R49ab348a2ce94d88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="4" r:id="R5871f94624c24805"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14508,16 +14508,16 @@
       <x:c r="C449" s="3" t="s">
         <x:v>473</x:v>
       </x:c>
-      <x:c r="D449" s="5">
-        <x:v>36106</x:v>
+      <x:c r="D449" s="5" t="n">
+        <x:v>36837</x:v>
       </x:c>
       <x:c r="E449" s="5">
         <x:v>43210</x:v>
       </x:c>
-      <x:c r="F449" s="1">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="G449" s="1">
+      <x:c r="F449" s="1" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G449" s="1" t="n">
         <x:v>164</x:v>
       </x:c>
     </x:row>
@@ -15934,16 +15934,16 @@
       <x:c r="C511" s="3" t="s">
         <x:v>546</x:v>
       </x:c>
-      <x:c r="D511" s="5">
-        <x:v>36648</x:v>
+      <x:c r="D511" s="5" t="n">
+        <x:v>36282</x:v>
       </x:c>
       <x:c r="E511" s="5">
         <x:v>43763</x:v>
       </x:c>
-      <x:c r="F511" s="1">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="G511" s="1">
+      <x:c r="F511" s="1" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G511" s="1" t="n">
         <x:v>176</x:v>
       </x:c>
     </x:row>
@@ -18188,16 +18188,16 @@
       <x:c r="C609" s="3" t="s">
         <x:v>661</x:v>
       </x:c>
-      <x:c r="D609" s="5">
-        <x:v>37924</x:v>
+      <x:c r="D609" s="5" t="n">
+        <x:v>37559</x:v>
       </x:c>
       <x:c r="E609" s="5">
         <x:v>44836</x:v>
       </x:c>
-      <x:c r="F609" s="1">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="G609" s="1">
+      <x:c r="F609" s="1" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G609" s="1" t="n">
         <x:v>337</x:v>
       </x:c>
     </x:row>
@@ -18924,8 +18924,8 @@
       <x:c r="C641" s="3" t="s">
         <x:v>697</x:v>
       </x:c>
-      <x:c r="D641" s="5">
-        <x:v>38526</x:v>
+      <x:c r="D641" s="5" t="n">
+        <x:v>38561</x:v>
       </x:c>
       <x:c r="E641" s="5">
         <x:v>45079</x:v>
@@ -18933,8 +18933,8 @@
       <x:c r="F641" s="1">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="G641" s="1">
-        <x:v>344</x:v>
+      <x:c r="G641" s="1" t="n">
+        <x:v>309</x:v>
       </x:c>
     </x:row>
     <x:row r="642">

</xml_diff>

<commit_message>
Adjust Yang Yuxin birth year
</commit_message>
<xml_diff>
--- a/SNH48成员名单生日表2603 (1).xlsx
+++ b/SNH48成员名单生日表2603 (1).xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="4" r:id="R5871f94624c24805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="4" r:id="R4eee733a7e604f8c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14509,13 +14509,13 @@
         <x:v>473</x:v>
       </x:c>
       <x:c r="D449" s="5" t="n">
-        <x:v>36837</x:v>
+        <x:v>35741</x:v>
       </x:c>
       <x:c r="E449" s="5">
         <x:v>43210</x:v>
       </x:c>
       <x:c r="F449" s="1" t="n">
-        <x:v>17</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G449" s="1" t="n">
         <x:v>164</x:v>

</xml_diff>